<commit_message>
Location of the sample added to the df
</commit_message>
<xml_diff>
--- a/testacce.xlsx
+++ b/testacce.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:AK6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,42 +446,167 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>ITS_length</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ITS_organism</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ITS_country</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ITS_collection_date</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ITS_voucher</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>rbcL_accession</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>rbcL_title</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>rbcL_length</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>rbcL_organism</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>rbcL_country</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>rbcL_collection_date</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>rbcL_voucher</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>matK_accession</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>matK_title</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>matK_length</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>matK_organism</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>matK_country</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>matK_collection_date</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>matK_voucher</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>trnL_accession</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>trnL_title</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>trnL_length</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>trnL_organism</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>trnL_country</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>trnL_collection_date</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>trnL_voucher</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>psbA-trnH_accession</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>psbA-trnH_title</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>psbA-trnH_length</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>psbA-trnH_organism</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>psbA-trnH_country</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>psbA-trnH_collection_date</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>psbA-trnH_voucher</t>
         </is>
       </c>
     </row>
@@ -496,44 +621,113 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
         <is>
           <t>PZ385908.1</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Huperzia selago voucher EDNA21-0061142 ribulose-1,5-bisphosphate carboxylase/oxygenase large subunit (rbcL) gene, partial cds; chloroplast</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="L2" t="n">
+        <v>607</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Huperzia selago</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>22-Jun-2021</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>EDNA21-0061142</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>NC_085757.1</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Huperzia selago voucher Hup20210022 chloroplast, complete genome</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="S2" t="n">
+        <v>161519</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Huperzia selago</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Hup20210022</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
         <is>
           <t>LT606116.1</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>Huperzia selago chloroplast genomic DNA containing trnL(UAA) intron region, isolate L1100-2-4 - Sequence 4</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="Z2" t="n">
+        <v>328</v>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Huperzia selago</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Jul-2015</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr">
         <is>
           <t>MW817416.1</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>Huperzia selago isolate 175 psbA-trnH intergenic spacer region, partial sequence; chloroplast</t>
+        </is>
+      </c>
+      <c r="AG2" t="n">
+        <v>303</v>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Huperzia selago</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>E.Oberndorfer s.n. (DUKE)</t>
         </is>
       </c>
     </row>
@@ -548,36 +742,87 @@
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>MW801557.1</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Lycopodiella inundata isolate 205 ribulose-1,5-bisphosphate carboxylase/oxygenase large subunit (rbcL) gene, partial cds; chloroplast</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>MW801557.1</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Lycopodiella inundata isolate 205 ribulose-1,5-bisphosphate carboxylase/oxygenase large subunit (rbcL) gene, partial cds; chloroplast</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>1248</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Lycopodiella inundata</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>A.Larsson AL750 (UPS)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr">
         <is>
           <t>MG560711.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>Lycopodiella inundata trnL-trnF intergenic spacer region, partial sequence; chloroplast</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="Z3" t="n">
+        <v>499</v>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Lycopodiella inundata</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr">
         <is>
           <t>MW817445.1</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="AF3" t="inlineStr">
         <is>
           <t>Lycopodiella inundata isolate 204 psbA-trnH intergenic spacer region, partial sequence; chloroplast</t>
+        </is>
+      </c>
+      <c r="AG3" t="n">
+        <v>295</v>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>Lycopodiella inundata</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>A.Larsson AL750 (UPS)</t>
         </is>
       </c>
     </row>
@@ -592,44 +837,109 @@
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>PV007079.1</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Lycopodium clavatum voucher Daniel Tejero-Diez 5868 (MEXU, US) ribulose-1,5-bisphosphate carboxylase/oxygenase large subunit (rbcL) gene, partial cds; chloroplast</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="L4" t="n">
+        <v>606</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Lycopodium clavatum</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Daniel Tejero-Diez 5868 (MEXU, US)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>PQ393062.1</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Lycopodium clavatum voucher KS23 HER0387 maturase K (matK) gene, partial cds; chloroplast</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="S4" t="n">
+        <v>437</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Lycopodium clavatum</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>KS23 HER0387</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t>PZ267855.1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>Lycopodium clavatum isolate LYCL tRNA-Leu (trnL) gene, intron; chloroplast</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="Z4" t="n">
+        <v>466</v>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Lycopodium clavatum</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>01-Jul-2020</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr">
         <is>
           <t>OQ309346.1</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>UNVERIFIED: Lycopodium clavatum voucher Eric Schuettpelz 1652 (MEXU, US) psbA-trnH intergenic spacer, partial sequence; chloroplast</t>
+        </is>
+      </c>
+      <c r="AG4" t="n">
+        <v>293</v>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Lycopodium clavatum</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>Eric Schuettpelz 1652 (MEXU, US)</t>
         </is>
       </c>
     </row>
@@ -644,44 +954,105 @@
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
         <is>
           <t>PQ435785.1</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Spinulum annotinum voucher KS23 HER0488 ribulose-1,5-bisphosphate carboxylase/oxygenase large subunit (rbcL) gene, partial cds; chloroplast</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="L5" t="n">
+        <v>281</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Spinulum annotinum</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>KS23 HER0488</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>PQ421744.1</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>Spinulum annotinum voucher KS23 HER0488 maturase K (matK) gene, partial cds; chloroplast</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="S5" t="n">
+        <v>361</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Spinulum annotinum</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>KS23 HER0488</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
         <is>
           <t>KF977453.1</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>Lycopodium annotinum trnL-F intergenic spacer, partial sequence; chloroplast</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="Z5" t="n">
+        <v>441</v>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>Spinulum annotinum</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr">
         <is>
           <t>MW817527.1</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="AF5" t="inlineStr">
         <is>
           <t>Spinulum annotinum isolate 286 psbA-trnH intergenic spacer region, partial sequence; chloroplast</t>
+        </is>
+      </c>
+      <c r="AG5" t="n">
+        <v>221</v>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>Spinulum annotinum</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>DJY04804 (CDBI)</t>
         </is>
       </c>
     </row>
@@ -696,210 +1067,119 @@
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
         <is>
           <t>PZ385972.1</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Diphasiastrum alpinum voucher EDNA21-0061143 ribulose-1,5-bisphosphate carboxylase/oxygenase large subunit (rbcL) gene, partial cds; chloroplast</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="L6" t="n">
+        <v>607</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Diphasiastrum alpinum</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>22-Jun-2021</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>EDNA21-0061143</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>MF953527.1</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>Diphasiastrum alpinum isolate DA3 maturase K (matK) gene, partial cds; chloroplast</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="S6" t="n">
+        <v>780</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Diphasiastrum alpinum</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>09-Jul-2013</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>VA21621</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
         <is>
           <t>PZ267825.1</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>Diphasiastrum alpinum isolate DIAL tRNA-Leu (trnL) gene, intron; chloroplast</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="Z6" t="n">
+        <v>455</v>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Diphasiastrum alpinum</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>01-Jul-2020</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr">
         <is>
           <t>MW817355.1</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="AF6" t="inlineStr">
         <is>
           <t>Diphasiastrum alpinum isolate 114 psbA-trnH intergenic spacer region, partial sequence; chloroplast</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Lycopodium issleri</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>MH064684.1</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Diphasiastrum issleri rbcL-atpB intergenic spacer, partial sequence; and ATP synthase CF1 beta subunit (atpB) gene, partial cds; chloroplast</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Lycopodium complanatum</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>OR188966.1</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Diphasiastrum complanatum voucher 765154 LabNo 1297 rbcL-atpB intergenic spacer, partial sequence; and ATP synthase CF1 beta subunit (atpB) gene, partial cds; chloroplast</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>MW817357.1</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Diphasiastrum complanatum isolate 116 psbA-trnH intergenic spacer region, partial sequence; chloroplast</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Lycopodium zeilleri</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>MH064724.1</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Diphasiastrum zeilleri rbcL-atpB intergenic spacer, partial sequence; and ATP synthase CF1 beta subunit (atpB) gene, partial cds; chloroplast</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Lycopodium tristachyum</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>MK526147.1</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Diphasiastrum tristachyum ribulose-1,5-bisphosphate carboxylase/oxygenase large subunit (rbcL) gene, partial cds; chloroplast</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>MG560701.1</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Diphasiastrum tristachyum trnL-trnF intergenic spacer region, partial sequence; chloroplast</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Isoetes lacustris</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>OM692074.1</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Isoetes lacustris voucher Tihimorov, Prokopova &amp; Samarina 11060 (C) ribulose-1,5-bisphosphate carboxylase/oxygenase large subunit (rbcL) gene, partial cds; plastid</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>AY651835.1</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Isoetes lacustris isolate CR005 tRNA-Leu gene and trnL-trnF intergenic spacer, partial sequence; chloroplast</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="AG6" t="n">
+        <v>279</v>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>Diphasiastrum alpinum</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>V.Reeb 8-VIII-02/3 (DUKE)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>